<commit_message>
Update lookup and reference function.xlsx
</commit_message>
<xml_diff>
--- a/lookup and reference function.xlsx
+++ b/lookup and reference function.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\M.D ZAKI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Zaki DA\Excel-Data-Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686AD087-83B9-4175-AC51-62BAFBF6CF61}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF5BF53F-E956-4A9A-B2C5-966CF5E4D84F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7005" xr2:uid="{01A7706D-DEF4-4A01-9BAB-A5C2388E7096}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7005" activeTab="2" xr2:uid="{01A7706D-DEF4-4A01-9BAB-A5C2388E7096}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="New Data" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="93">
   <si>
     <t>The Alchemist</t>
   </si>
@@ -296,6 +297,15 @@
   </si>
   <si>
     <t>Delhi</t>
+  </si>
+  <si>
+    <t>Kya be</t>
+  </si>
+  <si>
+    <t xml:space="preserve">So </t>
+  </si>
+  <si>
+    <t>Mat</t>
   </si>
 </sst>
 </file>
@@ -3658,4 +3668,29 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9150C93-8604-49DB-9227-6D8665B1B6FB}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>